<commit_message>
Alte Songs: Spalte "Neuer Vorschlag (KI)" mit Ideen je Part in 18 Tabellen
songgen.py --vorschlag schreibt die Texte aus songs/<Song>/vorschlag.yaml
über struktur.write_proposals() in die Tabelle (Kopie schreiben, zurücklesen,
nur ersetzen wenn sonst alles gleich ist). Die Spalte ist reine Ausgabe:
kein Song neu generiert, keine Show geändert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/BeMine_v1/quelle/struktur.xlsx
+++ b/songs/BeMine_v1/quelle/struktur.xlsx
@@ -438,16 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +473,7 @@
         <v>26</v>
       </c>
       <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -483,6 +485,7 @@
         <v>126</v>
       </c>
       <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -494,6 +497,7 @@
         <v>0.375</v>
       </c>
       <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -518,15 +522,20 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>Neuer Vorschlag (KI)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>Energie 0-5</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>BPM pro Part</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>bisher (alter Code)</t>
         </is>
@@ -548,12 +557,13 @@
         </is>
       </c>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>progBlack(5000, 5)   (Matrix: progScrollText("Be Mine by Kamrad", 20238, 75, getRandomColor(), 10))</t>
         </is>
@@ -575,12 +585,17 @@
         </is>
       </c>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Szene Glow, SUNSET, weich eingeblendet (fade_in 4 Beats).</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>progBlingBlingColoring(15238, 10, 946)</t>
         </is>
@@ -602,12 +617,17 @@
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Szene Verse, SUNSET: dezenter Puls im Beat (bisher Regenbogen-Streifen).</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>progPalette(15238, 1, 12)</t>
         </is>
@@ -629,12 +649,17 @@
         </is>
       </c>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Szene Palette, SUNSET -&gt; Farbwanderung nach NEON (2 Takte): Farbband über die ganze Bühne.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>progPalette(15238, 4, 14)</t>
         </is>
@@ -656,12 +681,17 @@
         </is>
       </c>
       <c r="D10" s="6" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Linien bleiben (stapeln sich), darüber baut sich ein Glitzern auf (Ebene Sparkle, fade_in über 7 Takte). Fester Look für beide.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>progRandomLines(13333, 16, 470, false)</t>
         </is>
@@ -683,12 +713,17 @@
         </is>
       </c>
       <c r="D11" s="6" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Szene Buildup (1 Takt), NEON: lädt sich auf, Explosion genau auf den Chorus - der Blinder des Users steht dann auf dem Einsatz.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>progFastBlingBling(1905, 6, 18)</t>
         </is>
@@ -715,12 +750,17 @@
           <t>starker blinder am Anfang!</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Szene Colors, NEON, soft 30 (feste Farben, kurze Blende); Blinder am Anfang bleibt. Auf der Matrix "BE MINE" über der Szene (2 Takte, blendet aus).</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>progFullColors(15238, 20, 470)</t>
         </is>
@@ -742,12 +782,17 @@
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Schwarz bleibt; in den letzten 2 Beats weich ins Verse (verse 2 mit Übergang fade).</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>progBlack(1905, 22)</t>
         </is>
@@ -769,12 +814,17 @@
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Leuchtspuren bleiben (Szene Rain, ROYAL) - kühler Kontrast zum Chorus.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>progMatrixHorizontal(15238, 24, 70, true)</t>
         </is>
@@ -796,12 +846,17 @@
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Szene DNA Flip, NEON: stehende Helix auf der Matrix, alle anderen pulsieren einmal je Takt (bisher Wasserringe).</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>progWaterRipple(15238, 26, 50, true, true)</t>
         </is>
@@ -823,12 +878,13 @@
         </is>
       </c>
       <c r="D16" s="6" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>progRandomLines(13333, 28, 470, false)</t>
         </is>
@@ -850,12 +906,17 @@
         </is>
       </c>
       <c r="D17" s="6" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>wie beim ersten Mal (Buildup).</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>progFastBlingBling(1905, 6, 30)</t>
         </is>
@@ -877,12 +938,17 @@
         </is>
       </c>
       <c r="D18" s="6" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Colors wie chorus 1, Blinder auf den Einsatz, Lampen blitzen weiß auf 2 und 4.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>progFullColors(13333, 32, 474)</t>
         </is>
@@ -904,12 +970,17 @@
         </is>
       </c>
       <c r="D19" s="6" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Starker Blinder statt Strobo: blendet 2 Beats ein und steht 2 Beats voll bis zum Einsatz von chorus 3.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>progStrobo(1905, 34, 120, 255, 255, 255)</t>
         </is>
@@ -936,12 +1007,17 @@
           <t>blinder am ende</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Anwachsende Einzelblitze bleiben, in FIRE; drei kurze Blinder Ende des 4. Takts (Takt 80,5 / 80,75 / 81). Der Blinder am Ende bleibt.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>progFastBlingBling(15238, 2, 36, 1, 20, 946)</t>
         </is>
@@ -961,10 +1037,10 @@
           <t>10 sek. BLACK</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <f>$C$3</f>
         <v/>
       </c>

</xml_diff>